<commit_message>
updated hospital example solution file
</commit_message>
<xml_diff>
--- a/assets/sheets/HospitalExampleSolutions.xlsx
+++ b/assets/sheets/HospitalExampleSolutions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10512"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/laurennelsen/Dropbox/UCCS/Teaching/QUAN 2010/PreTeXt files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BC5F226-9422-C547-8A79-AA3CD3B16D9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{951CEC1C-4C59-9E43-8C27-3750FD59767E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32800" yWindow="2440" windowWidth="26040" windowHeight="14940" xr2:uid="{026E9C3C-F9D3-9C47-A3CF-682EAB19F009}"/>
+    <workbookView xWindow="8120" yWindow="760" windowWidth="22120" windowHeight="17860" xr2:uid="{026E9C3C-F9D3-9C47-A3CF-682EAB19F009}"/>
   </bookViews>
   <sheets>
     <sheet name="HospitalExample" sheetId="1" r:id="rId1"/>
@@ -221,14 +221,14 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1141,16 +1141,16 @@
       <c r="D24" s="3">
         <v>0</v>
       </c>
-      <c r="F24" s="7" t="s">
+      <c r="F24" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="G24" s="7"/>
-      <c r="H24" s="7"/>
-      <c r="I24" s="7"/>
-      <c r="J24" s="7"/>
-      <c r="K24" s="7"/>
-      <c r="L24" s="7"/>
-      <c r="M24" s="7"/>
+      <c r="G24" s="9"/>
+      <c r="H24" s="9"/>
+      <c r="I24" s="9"/>
+      <c r="J24" s="9"/>
+      <c r="K24" s="9"/>
+      <c r="L24" s="9"/>
+      <c r="M24" s="9"/>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A25" s="2">
@@ -1165,14 +1165,14 @@
       <c r="D25" s="3">
         <v>0</v>
       </c>
-      <c r="F25" s="7"/>
-      <c r="G25" s="7"/>
-      <c r="H25" s="7"/>
-      <c r="I25" s="7"/>
-      <c r="J25" s="7"/>
-      <c r="K25" s="7"/>
-      <c r="L25" s="7"/>
-      <c r="M25" s="7"/>
+      <c r="F25" s="9"/>
+      <c r="G25" s="9"/>
+      <c r="H25" s="9"/>
+      <c r="I25" s="9"/>
+      <c r="J25" s="9"/>
+      <c r="K25" s="9"/>
+      <c r="L25" s="9"/>
+      <c r="M25" s="9"/>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A26" s="2">
@@ -1187,14 +1187,14 @@
       <c r="D26" s="3">
         <v>0</v>
       </c>
-      <c r="F26" s="7"/>
-      <c r="G26" s="7"/>
-      <c r="H26" s="7"/>
-      <c r="I26" s="7"/>
-      <c r="J26" s="7"/>
-      <c r="K26" s="7"/>
-      <c r="L26" s="7"/>
-      <c r="M26" s="7"/>
+      <c r="F26" s="9"/>
+      <c r="G26" s="9"/>
+      <c r="H26" s="9"/>
+      <c r="I26" s="9"/>
+      <c r="J26" s="9"/>
+      <c r="K26" s="9"/>
+      <c r="L26" s="9"/>
+      <c r="M26" s="9"/>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A27" s="2">
@@ -1209,16 +1209,16 @@
       <c r="D27" s="3">
         <v>1</v>
       </c>
-      <c r="F27" s="7" t="s">
+      <c r="F27" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="G27" s="7"/>
-      <c r="H27" s="7"/>
-      <c r="I27" s="7"/>
-      <c r="J27" s="7"/>
-      <c r="K27" s="7"/>
-      <c r="L27" s="7"/>
-      <c r="M27" s="7"/>
+      <c r="G27" s="9"/>
+      <c r="H27" s="9"/>
+      <c r="I27" s="9"/>
+      <c r="J27" s="9"/>
+      <c r="K27" s="9"/>
+      <c r="L27" s="9"/>
+      <c r="M27" s="9"/>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A28" s="2">
@@ -1233,14 +1233,14 @@
       <c r="D28" s="3">
         <v>0</v>
       </c>
-      <c r="F28" s="7"/>
-      <c r="G28" s="7"/>
-      <c r="H28" s="7"/>
-      <c r="I28" s="7"/>
-      <c r="J28" s="7"/>
-      <c r="K28" s="7"/>
-      <c r="L28" s="7"/>
-      <c r="M28" s="7"/>
+      <c r="F28" s="9"/>
+      <c r="G28" s="9"/>
+      <c r="H28" s="9"/>
+      <c r="I28" s="9"/>
+      <c r="J28" s="9"/>
+      <c r="K28" s="9"/>
+      <c r="L28" s="9"/>
+      <c r="M28" s="9"/>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A29" s="2">
@@ -1258,25 +1258,25 @@
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A30" s="2">
-        <v>10775</v>
+        <v>10596</v>
       </c>
       <c r="B30" s="3">
-        <v>72</v>
+        <v>24</v>
       </c>
       <c r="C30" s="3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D30" s="3">
         <v>0</v>
       </c>
-      <c r="H30" s="8"/>
+      <c r="H30" s="7"/>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A31" s="2">
-        <v>12215</v>
+        <v>10775</v>
       </c>
       <c r="B31" s="3">
-        <v>35</v>
+        <v>72</v>
       </c>
       <c r="C31" s="3">
         <v>4</v>
@@ -1284,72 +1284,72 @@
       <c r="D31" s="3">
         <v>0</v>
       </c>
-      <c r="G31" s="9"/>
-      <c r="H31" s="9"/>
-      <c r="I31" s="9"/>
-      <c r="J31" s="9"/>
-      <c r="K31" s="9"/>
-      <c r="L31" s="9"/>
-      <c r="M31" s="9"/>
+      <c r="G31" s="10"/>
+      <c r="H31" s="10"/>
+      <c r="I31" s="10"/>
+      <c r="J31" s="10"/>
+      <c r="K31" s="10"/>
+      <c r="L31" s="10"/>
+      <c r="M31" s="10"/>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A32" s="2">
-        <v>12419</v>
+        <v>12215</v>
       </c>
       <c r="B32" s="3">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="C32" s="3">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D32" s="3">
         <v>0</v>
       </c>
-      <c r="G32" s="9"/>
-      <c r="H32" s="9"/>
-      <c r="I32" s="9"/>
-      <c r="J32" s="9"/>
-      <c r="K32" s="9"/>
-      <c r="L32" s="9"/>
-      <c r="M32" s="9"/>
+      <c r="G32" s="10"/>
+      <c r="H32" s="10"/>
+      <c r="I32" s="10"/>
+      <c r="J32" s="10"/>
+      <c r="K32" s="10"/>
+      <c r="L32" s="10"/>
+      <c r="M32" s="10"/>
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A33" s="2">
-        <v>12592</v>
+        <v>12419</v>
       </c>
       <c r="B33" s="3">
-        <v>29</v>
+        <v>46</v>
       </c>
       <c r="C33" s="3">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D33" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A34" s="2">
-        <v>12621</v>
+        <v>12592</v>
       </c>
       <c r="B34" s="3">
-        <v>75</v>
+        <v>29</v>
       </c>
       <c r="C34" s="3">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D34" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A35" s="2">
-        <v>13034</v>
+        <v>12621</v>
       </c>
       <c r="B35" s="3">
-        <v>36</v>
+        <v>75</v>
       </c>
       <c r="C35" s="3">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D35" s="3">
         <v>0</v>
@@ -1357,10 +1357,10 @@
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A36" s="2">
-        <v>13281</v>
+        <v>13034</v>
       </c>
       <c r="B36" s="3">
-        <v>81</v>
+        <v>36</v>
       </c>
       <c r="C36" s="3">
         <v>6</v>
@@ -1371,159 +1371,159 @@
     </row>
     <row r="37" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A37" s="2">
-        <v>13580</v>
+        <v>13281</v>
       </c>
       <c r="B37" s="3">
-        <v>69</v>
+        <v>81</v>
       </c>
       <c r="C37" s="3">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D37" s="3">
-        <v>1</v>
-      </c>
-      <c r="G37" s="7"/>
-      <c r="H37" s="7"/>
-      <c r="I37" s="7"/>
-      <c r="J37" s="7"/>
-      <c r="K37" s="7"/>
-      <c r="L37" s="7"/>
-      <c r="M37" s="7"/>
-      <c r="N37" s="7"/>
+        <v>0</v>
+      </c>
+      <c r="G37" s="9"/>
+      <c r="H37" s="9"/>
+      <c r="I37" s="9"/>
+      <c r="J37" s="9"/>
+      <c r="K37" s="9"/>
+      <c r="L37" s="9"/>
+      <c r="M37" s="9"/>
+      <c r="N37" s="9"/>
     </row>
     <row r="38" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A38" s="2">
-        <v>13647</v>
+        <v>13580</v>
       </c>
       <c r="B38" s="3">
-        <v>35</v>
+        <v>69</v>
       </c>
       <c r="C38" s="3">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D38" s="3">
-        <v>0</v>
-      </c>
-      <c r="G38" s="7"/>
-      <c r="H38" s="7"/>
-      <c r="I38" s="7"/>
-      <c r="J38" s="7"/>
-      <c r="K38" s="7"/>
-      <c r="L38" s="7"/>
-      <c r="M38" s="7"/>
-      <c r="N38" s="7"/>
+        <v>1</v>
+      </c>
+      <c r="G38" s="9"/>
+      <c r="H38" s="9"/>
+      <c r="I38" s="9"/>
+      <c r="J38" s="9"/>
+      <c r="K38" s="9"/>
+      <c r="L38" s="9"/>
+      <c r="M38" s="9"/>
+      <c r="N38" s="9"/>
     </row>
     <row r="39" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A39" s="2">
-        <v>18457</v>
+        <v>13647</v>
       </c>
       <c r="B39" s="3">
-        <v>53</v>
+        <v>35</v>
       </c>
       <c r="C39" s="3">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="D39" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A40" s="2">
-        <v>16978</v>
+        <v>18457</v>
       </c>
       <c r="B40" s="3">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C40" s="3">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="D40" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="41" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A41" s="2">
-        <v>18392</v>
+        <v>16978</v>
       </c>
       <c r="B41" s="3">
-        <v>41</v>
+        <v>56</v>
       </c>
       <c r="C41" s="3">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D41" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A42" s="2">
-        <v>18759</v>
+        <v>18392</v>
       </c>
       <c r="B42" s="3">
-        <v>87</v>
+        <v>41</v>
       </c>
       <c r="C42" s="3">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D42" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A43" s="2">
-        <v>17393</v>
+        <v>18759</v>
       </c>
       <c r="B43" s="3">
-        <v>51</v>
+        <v>87</v>
       </c>
       <c r="C43" s="3">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D43" s="3">
-        <v>2</v>
-      </c>
-      <c r="G43" s="7"/>
-      <c r="H43" s="7"/>
-      <c r="I43" s="7"/>
-      <c r="J43" s="7"/>
-      <c r="K43" s="7"/>
-      <c r="L43" s="7"/>
-      <c r="M43" s="7"/>
-      <c r="N43" s="7"/>
-      <c r="O43" s="7"/>
+        <v>0</v>
+      </c>
+      <c r="G43" s="9"/>
+      <c r="H43" s="9"/>
+      <c r="I43" s="9"/>
+      <c r="J43" s="9"/>
+      <c r="K43" s="9"/>
+      <c r="L43" s="9"/>
+      <c r="M43" s="9"/>
+      <c r="N43" s="9"/>
+      <c r="O43" s="9"/>
     </row>
     <row r="44" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A44" s="2">
-        <v>20554</v>
+        <v>17393</v>
       </c>
       <c r="B44" s="3">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C44" s="3">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D44" s="3">
-        <v>0</v>
-      </c>
-      <c r="G44" s="7"/>
-      <c r="H44" s="7"/>
-      <c r="I44" s="7"/>
-      <c r="J44" s="7"/>
-      <c r="K44" s="7"/>
-      <c r="L44" s="7"/>
-      <c r="M44" s="7"/>
-      <c r="N44" s="7"/>
-      <c r="O44" s="7"/>
+        <v>2</v>
+      </c>
+      <c r="G44" s="9"/>
+      <c r="H44" s="9"/>
+      <c r="I44" s="9"/>
+      <c r="J44" s="9"/>
+      <c r="K44" s="9"/>
+      <c r="L44" s="9"/>
+      <c r="M44" s="9"/>
+      <c r="N44" s="9"/>
+      <c r="O44" s="9"/>
     </row>
     <row r="45" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A45" s="2">
-        <v>14560</v>
+        <v>20554</v>
       </c>
       <c r="B45" s="3">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="C45" s="3">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="D45" s="3">
         <v>0</v>
@@ -1531,143 +1531,155 @@
     </row>
     <row r="46" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A46" s="2">
-        <v>28596</v>
+        <v>14560</v>
       </c>
       <c r="B46" s="3">
-        <v>57</v>
+        <v>38</v>
       </c>
       <c r="C46" s="3">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D46" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A47" s="2">
-        <v>28804</v>
+        <v>28596</v>
       </c>
       <c r="B47" s="3">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="C47" s="3">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="D47" s="3">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A48" s="2">
-        <v>22514</v>
+        <v>28804</v>
       </c>
       <c r="B48" s="3">
-        <v>51</v>
+        <v>62</v>
       </c>
       <c r="C48" s="3">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="D48" s="3">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="49" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A49" s="2">
-        <v>32660</v>
+        <v>22514</v>
       </c>
       <c r="B49" s="3">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C49" s="3">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="D49" s="3">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A50" s="2">
+        <v>32660</v>
+      </c>
+      <c r="B50" s="3">
+        <v>49</v>
+      </c>
+      <c r="C50" s="3">
+        <v>14</v>
+      </c>
+      <c r="D50" s="3">
+        <v>3</v>
+      </c>
+      <c r="G50" s="9"/>
+      <c r="H50" s="9"/>
+      <c r="I50" s="9"/>
+      <c r="J50" s="9"/>
+      <c r="K50" s="9"/>
+      <c r="L50" s="9"/>
+      <c r="M50" s="9"/>
+      <c r="N50" s="9"/>
+      <c r="O50" s="9"/>
+    </row>
+    <row r="51" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A51" s="2">
         <v>34460</v>
       </c>
-      <c r="B50" s="3">
+      <c r="B51" s="3">
         <v>71</v>
       </c>
-      <c r="C50" s="3">
+      <c r="C51" s="3">
         <v>10</v>
       </c>
-      <c r="D50" s="3">
+      <c r="D51" s="3">
         <v>2</v>
       </c>
-      <c r="G50" s="7"/>
-      <c r="H50" s="7"/>
-      <c r="I50" s="7"/>
-      <c r="J50" s="7"/>
-      <c r="K50" s="7"/>
-      <c r="L50" s="7"/>
-      <c r="M50" s="7"/>
-      <c r="N50" s="7"/>
-      <c r="O50" s="7"/>
-    </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="G51" s="7"/>
-      <c r="H51" s="7"/>
-      <c r="I51" s="7"/>
-      <c r="J51" s="7"/>
-      <c r="K51" s="7"/>
-      <c r="L51" s="7"/>
-      <c r="M51" s="7"/>
-      <c r="N51" s="7"/>
-      <c r="O51" s="7"/>
+      <c r="G51" s="9"/>
+      <c r="H51" s="9"/>
+      <c r="I51" s="9"/>
+      <c r="J51" s="9"/>
+      <c r="K51" s="9"/>
+      <c r="L51" s="9"/>
+      <c r="M51" s="9"/>
+      <c r="N51" s="9"/>
+      <c r="O51" s="9"/>
     </row>
     <row r="57" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="G57" s="7"/>
-      <c r="H57" s="7"/>
-      <c r="I57" s="7"/>
-      <c r="J57" s="7"/>
-      <c r="K57" s="7"/>
-      <c r="L57" s="7"/>
-      <c r="M57" s="7"/>
-      <c r="N57" s="7"/>
-      <c r="O57" s="7"/>
+      <c r="G57" s="9"/>
+      <c r="H57" s="9"/>
+      <c r="I57" s="9"/>
+      <c r="J57" s="9"/>
+      <c r="K57" s="9"/>
+      <c r="L57" s="9"/>
+      <c r="M57" s="9"/>
+      <c r="N57" s="9"/>
+      <c r="O57" s="9"/>
     </row>
     <row r="58" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="G58" s="7"/>
-      <c r="H58" s="7"/>
-      <c r="I58" s="7"/>
-      <c r="J58" s="7"/>
-      <c r="K58" s="7"/>
-      <c r="L58" s="7"/>
-      <c r="M58" s="7"/>
-      <c r="N58" s="7"/>
-      <c r="O58" s="7"/>
+      <c r="G58" s="9"/>
+      <c r="H58" s="9"/>
+      <c r="I58" s="9"/>
+      <c r="J58" s="9"/>
+      <c r="K58" s="9"/>
+      <c r="L58" s="9"/>
+      <c r="M58" s="9"/>
+      <c r="N58" s="9"/>
+      <c r="O58" s="9"/>
     </row>
     <row r="61" spans="1:15" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="I61" s="7"/>
-      <c r="J61" s="7"/>
-      <c r="K61" s="7"/>
-      <c r="L61" s="7"/>
-      <c r="M61" s="7"/>
-      <c r="N61" s="7"/>
-      <c r="O61" s="7"/>
+      <c r="I61" s="9"/>
+      <c r="J61" s="9"/>
+      <c r="K61" s="9"/>
+      <c r="L61" s="9"/>
+      <c r="M61" s="9"/>
+      <c r="N61" s="9"/>
+      <c r="O61" s="9"/>
     </row>
     <row r="62" spans="1:15" ht="39" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="I62" s="7"/>
-      <c r="J62" s="7"/>
-      <c r="K62" s="7"/>
-      <c r="L62" s="7"/>
-      <c r="M62" s="7"/>
-      <c r="N62" s="7"/>
-      <c r="O62" s="7"/>
+      <c r="I62" s="9"/>
+      <c r="J62" s="9"/>
+      <c r="K62" s="9"/>
+      <c r="L62" s="9"/>
+      <c r="M62" s="9"/>
+      <c r="N62" s="9"/>
+      <c r="O62" s="9"/>
     </row>
     <row r="63" spans="1:15" ht="35.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="G63" s="10"/>
-      <c r="I63" s="7"/>
-      <c r="J63" s="7"/>
-      <c r="K63" s="7"/>
-      <c r="L63" s="7"/>
-      <c r="M63" s="7"/>
-      <c r="N63" s="7"/>
-      <c r="O63" s="7"/>
+      <c r="G63" s="8"/>
+      <c r="I63" s="9"/>
+      <c r="J63" s="9"/>
+      <c r="K63" s="9"/>
+      <c r="L63" s="9"/>
+      <c r="M63" s="9"/>
+      <c r="N63" s="9"/>
+      <c r="O63" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="10">

</xml_diff>